<commit_message>
Finalize published analytics deliverables
</commit_message>
<xml_diff>
--- a/documentation/University_Data_Dictionary.xlsx
+++ b/documentation/University_Data_Dictionary.xlsx
@@ -778,10 +778,10 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>320</v>
+        <v>1000</v>
       </c>
       <c r="F13" t="n">
-        <v>680</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">

</xml_diff>